<commit_message>
Refactor SQL analysis scripts and documentation for Malang Food Analysis project
- Updated database schema to include primary key and improved comments.
- Revised import instructions for clarity and added validation steps.
- Removed outdated query result files and replaced them with new structured output files.
- Enhanced SQL queries for better readability and added new exploratory queries.
- Documented learning journey in SQL and Python, focusing on data analysis techniques.
- Added new query results files for detailed insights on menu categories, pricing, and reviews.
</commit_message>
<xml_diff>
--- a/data/raw/Malang_City_Food_Record_Dataset_By_Google_Maps.xlsx
+++ b/data/raw/Malang_City_Food_Record_Dataset_By_Google_Maps.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\malang-food-analysis\data\raw\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Fahrul Fauji\06_Portofolio\malang-food-analysis\data\raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB5F78D6-3C4E-40DE-BE9D-15D18DC62EEA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{39361586-7140-4638-8A26-0401AAAEA63A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="330" windowWidth="20730" windowHeight="11310" xr2:uid="{EB3429D4-445B-4229-9669-062A08EA2914}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" xr2:uid="{EB3429D4-445B-4229-9669-062A08EA2914}"/>
   </bookViews>
   <sheets>
     <sheet name="Dataset_Kota_Malang" sheetId="1" r:id="rId1"/>
@@ -871,19 +871,19 @@
   </cellStyleXfs>
   <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="1" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -901,106 +901,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>374</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>3324224</xdr:colOff>
-      <xdr:row>378</xdr:row>
-      <xdr:rowOff>85726</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="2" name="TextBox 1">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{9C78F8A9-CAE2-4372-8DFF-4A1521E27A3F}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvSpPr txBox="1"/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="609600" y="75999975"/>
-          <a:ext cx="3324224" cy="847726"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:solidFill>
-          <a:schemeClr val="accent4">
-            <a:lumMod val="60000"/>
-            <a:lumOff val="40000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:ln w="9525" cmpd="sng">
-          <a:solidFill>
-            <a:schemeClr val="lt1">
-              <a:shade val="50000"/>
-            </a:schemeClr>
-          </a:solidFill>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:fillRef>
-        <a:effectRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="dk1"/>
-        </a:fontRef>
-      </xdr:style>
-      <xdr:txBody>
-        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:r>
-            <a:rPr lang="en-ID" sz="1200" b="1"/>
-            <a:t>Log Kegiatan :</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:r>
-            <a:rPr lang="en-ID" sz="1100"/>
-            <a:t>Dataset digabungkan di tanggal 29 september tahun 2025 jam 2:18</a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-ID" sz="1100" baseline="0"/>
-            <a:t> PM</a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-ID" sz="1100"/>
-            <a:t> dari Google</a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-ID" sz="1100" baseline="0"/>
-            <a:t> Maps</a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-ID" sz="1100"/>
-            <a:t>.</a:t>
-          </a:r>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1301,27 +1201,27 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{98A8680F-2210-408F-A3B7-DB84FF700D87}">
   <dimension ref="A1:I373"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="4.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="64.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15.5703125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="19.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="20.28515625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="19.7109375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="6.85546875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="14.5703125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="16.140625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="18.28515625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="18.28515625" customWidth="1"/>
-    <col min="12" max="12" width="28.85546875" bestFit="1" customWidth="1"/>
-    <col min="13" max="16" width="18.28515625" customWidth="1"/>
-    <col min="17" max="17" width="19.5703125" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="19.5703125" customWidth="1"/>
-    <col min="19" max="19" width="20.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="4.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="64.453125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.54296875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="19.1796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="20.26953125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="19.7265625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="6.81640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="14.54296875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="16.1796875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="18.26953125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="18.26953125" customWidth="1"/>
+    <col min="12" max="12" width="28.81640625" bestFit="1" customWidth="1"/>
+    <col min="13" max="16" width="18.26953125" customWidth="1"/>
+    <col min="17" max="17" width="19.54296875" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="19.54296875" customWidth="1"/>
+    <col min="19" max="19" width="20.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1350,7 +1250,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A2" s="2">
         <v>1</v>
       </c>
@@ -1379,7 +1279,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A3" s="2">
         <v>2</v>
       </c>
@@ -1408,7 +1308,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="4" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A4" s="2">
         <v>3</v>
       </c>
@@ -1437,7 +1337,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="5" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A5" s="2">
         <v>4</v>
       </c>
@@ -1466,7 +1366,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="6" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A6" s="2">
         <v>5</v>
       </c>
@@ -1495,7 +1395,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="7" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A7" s="2">
         <v>6</v>
       </c>
@@ -1524,7 +1424,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="8" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A8" s="2">
         <v>7</v>
       </c>
@@ -1553,7 +1453,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="9" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A9" s="2">
         <v>8</v>
       </c>
@@ -1582,7 +1482,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="10" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A10" s="2">
         <v>9</v>
       </c>
@@ -1611,7 +1511,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="11" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A11" s="2">
         <v>10</v>
       </c>
@@ -1640,7 +1540,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="12" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A12" s="2">
         <v>11</v>
       </c>
@@ -1669,7 +1569,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="13" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A13" s="2">
         <v>12</v>
       </c>
@@ -1698,7 +1598,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="14" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A14" s="2">
         <v>13</v>
       </c>
@@ -1727,7 +1627,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="15" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A15" s="2">
         <v>14</v>
       </c>
@@ -1756,7 +1656,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="16" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A16" s="2">
         <v>15</v>
       </c>
@@ -1785,7 +1685,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="17" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A17" s="2">
         <v>16</v>
       </c>
@@ -1814,7 +1714,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="18" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A18" s="2">
         <v>17</v>
       </c>
@@ -1843,7 +1743,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="19" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A19" s="2">
         <v>18</v>
       </c>
@@ -1872,7 +1772,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="20" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A20" s="2">
         <v>19</v>
       </c>
@@ -1901,7 +1801,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="21" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A21" s="2">
         <v>20</v>
       </c>
@@ -1930,7 +1830,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="22" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A22" s="2">
         <v>21</v>
       </c>
@@ -1959,7 +1859,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="23" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A23" s="2">
         <v>22</v>
       </c>
@@ -1988,7 +1888,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="24" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A24" s="2">
         <v>23</v>
       </c>
@@ -2017,7 +1917,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="25" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A25" s="2">
         <v>24</v>
       </c>
@@ -2046,7 +1946,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="26" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A26" s="2">
         <v>25</v>
       </c>
@@ -2075,7 +1975,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="27" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A27" s="2">
         <v>26</v>
       </c>
@@ -2104,7 +2004,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="28" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A28" s="2">
         <v>27</v>
       </c>
@@ -2133,7 +2033,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="29" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A29" s="2">
         <v>28</v>
       </c>
@@ -2162,7 +2062,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="30" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A30" s="2">
         <v>29</v>
       </c>
@@ -2191,7 +2091,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="31" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A31" s="2">
         <v>30</v>
       </c>
@@ -2220,7 +2120,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="32" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A32" s="2">
         <v>31</v>
       </c>
@@ -2249,7 +2149,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="33" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A33" s="2">
         <v>32</v>
       </c>
@@ -2278,7 +2178,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="34" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A34" s="2">
         <v>33</v>
       </c>
@@ -2307,7 +2207,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="35" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A35" s="2">
         <v>34</v>
       </c>
@@ -2336,7 +2236,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="36" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A36" s="2">
         <v>35</v>
       </c>
@@ -2365,7 +2265,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="37" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A37" s="2">
         <v>36</v>
       </c>
@@ -2394,7 +2294,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="38" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A38" s="2">
         <v>37</v>
       </c>
@@ -2423,7 +2323,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="39" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A39" s="2">
         <v>38</v>
       </c>
@@ -2452,7 +2352,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="40" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A40" s="2">
         <v>39</v>
       </c>
@@ -2481,7 +2381,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="41" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A41" s="2">
         <v>40</v>
       </c>
@@ -2510,7 +2410,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="42" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A42" s="2">
         <v>41</v>
       </c>
@@ -2539,7 +2439,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="43" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A43" s="2">
         <v>42</v>
       </c>
@@ -2568,7 +2468,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="44" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A44" s="2">
         <v>43</v>
       </c>
@@ -2597,7 +2497,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="45" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A45" s="2">
         <v>44</v>
       </c>
@@ -2626,7 +2526,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="46" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A46" s="2">
         <v>45</v>
       </c>
@@ -2655,7 +2555,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="47" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A47" s="2">
         <v>46</v>
       </c>
@@ -2684,7 +2584,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="48" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A48" s="2">
         <v>47</v>
       </c>
@@ -2713,7 +2613,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="49" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A49" s="2">
         <v>48</v>
       </c>
@@ -2742,7 +2642,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="50" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A50" s="2">
         <v>49</v>
       </c>
@@ -2771,7 +2671,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="51" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A51" s="2">
         <v>50</v>
       </c>
@@ -2800,7 +2700,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="52" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A52" s="2">
         <v>51</v>
       </c>
@@ -2829,7 +2729,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="53" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A53" s="2">
         <v>52</v>
       </c>
@@ -2858,7 +2758,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="54" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A54" s="2">
         <v>53</v>
       </c>
@@ -2887,7 +2787,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="55" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A55" s="2">
         <v>54</v>
       </c>
@@ -2916,7 +2816,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="56" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A56" s="2">
         <v>55</v>
       </c>
@@ -2945,7 +2845,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="57" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A57" s="2">
         <v>56</v>
       </c>
@@ -2974,7 +2874,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="58" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A58" s="2">
         <v>57</v>
       </c>
@@ -3003,7 +2903,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="59" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A59" s="2">
         <v>58</v>
       </c>
@@ -3032,7 +2932,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="60" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A60" s="2">
         <v>59</v>
       </c>
@@ -3061,7 +2961,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="61" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A61" s="2">
         <v>60</v>
       </c>
@@ -3090,7 +2990,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="62" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A62" s="2">
         <v>61</v>
       </c>
@@ -3119,7 +3019,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="63" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A63" s="2">
         <v>62</v>
       </c>
@@ -3148,7 +3048,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="64" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A64" s="2">
         <v>63</v>
       </c>
@@ -3177,7 +3077,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="65" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A65" s="2">
         <v>64</v>
       </c>
@@ -3206,7 +3106,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="66" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A66" s="2">
         <v>65</v>
       </c>
@@ -3235,7 +3135,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="67" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A67" s="2">
         <v>66</v>
       </c>
@@ -3264,7 +3164,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="68" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A68" s="2">
         <v>67</v>
       </c>
@@ -3293,7 +3193,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="69" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A69" s="2">
         <v>68</v>
       </c>
@@ -3322,7 +3222,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="70" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A70" s="2">
         <v>69</v>
       </c>
@@ -3351,7 +3251,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="71" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A71" s="2">
         <v>70</v>
       </c>
@@ -3380,7 +3280,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="72" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A72" s="2">
         <v>71</v>
       </c>
@@ -3409,7 +3309,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="73" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A73" s="2">
         <v>72</v>
       </c>
@@ -3438,7 +3338,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="74" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A74" s="2">
         <v>73</v>
       </c>
@@ -3467,7 +3367,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="75" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A75" s="2">
         <v>74</v>
       </c>
@@ -3496,7 +3396,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="76" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A76" s="2">
         <v>75</v>
       </c>
@@ -3525,7 +3425,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="77" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A77" s="2">
         <v>76</v>
       </c>
@@ -3554,7 +3454,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="78" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A78" s="2">
         <v>77</v>
       </c>
@@ -3583,7 +3483,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="79" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A79" s="2">
         <v>78</v>
       </c>
@@ -3612,7 +3512,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="80" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A80" s="2">
         <v>79</v>
       </c>
@@ -3641,7 +3541,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="81" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A81" s="2">
         <v>80</v>
       </c>
@@ -3670,7 +3570,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="82" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A82" s="2">
         <v>81</v>
       </c>
@@ -3699,7 +3599,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="83" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A83" s="2">
         <v>82</v>
       </c>
@@ -3728,7 +3628,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="84" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A84" s="2">
         <v>83</v>
       </c>
@@ -3757,7 +3657,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="85" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A85" s="2">
         <v>84</v>
       </c>
@@ -3786,7 +3686,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="86" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A86" s="2">
         <v>85</v>
       </c>
@@ -3815,7 +3715,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="87" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A87" s="2">
         <v>86</v>
       </c>
@@ -3844,7 +3744,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="88" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A88" s="2">
         <v>87</v>
       </c>
@@ -3873,7 +3773,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="89" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A89" s="2">
         <v>88</v>
       </c>
@@ -3902,7 +3802,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="90" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A90" s="2">
         <v>89</v>
       </c>
@@ -3931,7 +3831,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="91" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A91" s="2">
         <v>90</v>
       </c>
@@ -3960,7 +3860,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="92" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A92" s="2">
         <v>91</v>
       </c>
@@ -3989,7 +3889,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="93" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A93" s="2">
         <v>92</v>
       </c>
@@ -4018,7 +3918,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="94" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A94" s="2">
         <v>93</v>
       </c>
@@ -4047,7 +3947,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="95" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A95" s="2">
         <v>94</v>
       </c>
@@ -4076,7 +3976,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="96" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A96" s="2">
         <v>95</v>
       </c>
@@ -4105,7 +4005,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="97" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A97" s="2">
         <v>96</v>
       </c>
@@ -4134,7 +4034,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="98" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A98" s="2">
         <v>97</v>
       </c>
@@ -4163,7 +4063,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="99" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A99" s="2">
         <v>98</v>
       </c>
@@ -4192,7 +4092,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="100" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A100" s="2">
         <v>99</v>
       </c>
@@ -4221,7 +4121,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="101" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A101" s="2">
         <v>100</v>
       </c>
@@ -4250,7 +4150,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="102" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A102" s="2">
         <v>101</v>
       </c>
@@ -4279,7 +4179,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="103" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A103" s="2">
         <v>102</v>
       </c>
@@ -4308,7 +4208,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="104" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A104" s="2">
         <v>103</v>
       </c>
@@ -4337,7 +4237,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="105" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A105" s="2">
         <v>104</v>
       </c>
@@ -4366,7 +4266,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="106" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A106" s="2">
         <v>105</v>
       </c>
@@ -4395,7 +4295,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="107" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A107" s="2">
         <v>106</v>
       </c>
@@ -4424,7 +4324,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="108" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A108" s="2">
         <v>107</v>
       </c>
@@ -4453,7 +4353,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="109" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A109" s="2">
         <v>108</v>
       </c>
@@ -4482,7 +4382,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="110" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A110" s="2">
         <v>109</v>
       </c>
@@ -4511,7 +4411,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="111" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A111" s="2">
         <v>110</v>
       </c>
@@ -4540,7 +4440,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="112" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A112" s="2">
         <v>111</v>
       </c>
@@ -4569,7 +4469,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="113" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A113" s="2">
         <v>112</v>
       </c>
@@ -4598,7 +4498,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="114" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A114" s="2">
         <v>113</v>
       </c>
@@ -4627,7 +4527,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="115" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A115" s="2">
         <v>114</v>
       </c>
@@ -4656,7 +4556,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="116" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A116" s="2">
         <v>115</v>
       </c>
@@ -4685,7 +4585,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="117" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A117" s="2">
         <v>116</v>
       </c>
@@ -4714,7 +4614,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="118" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A118" s="2">
         <v>117</v>
       </c>
@@ -4743,7 +4643,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="119" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A119" s="2">
         <v>118</v>
       </c>
@@ -4772,7 +4672,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="120" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A120" s="2">
         <v>119</v>
       </c>
@@ -4801,7 +4701,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="121" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A121" s="2">
         <v>120</v>
       </c>
@@ -4830,7 +4730,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="122" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A122" s="2">
         <v>121</v>
       </c>
@@ -4859,7 +4759,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="123" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A123" s="2">
         <v>122</v>
       </c>
@@ -4888,7 +4788,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="124" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A124" s="2">
         <v>123</v>
       </c>
@@ -4917,7 +4817,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="125" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A125" s="2">
         <v>124</v>
       </c>
@@ -4946,7 +4846,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="126" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A126" s="2">
         <v>125</v>
       </c>
@@ -4975,7 +4875,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="127" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A127" s="2">
         <v>126</v>
       </c>
@@ -5004,7 +4904,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="128" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A128" s="2">
         <v>127</v>
       </c>
@@ -5033,7 +4933,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="129" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A129" s="2">
         <v>128</v>
       </c>
@@ -5062,7 +4962,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="130" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A130" s="2">
         <v>129</v>
       </c>
@@ -5091,7 +4991,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="131" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A131" s="2">
         <v>130</v>
       </c>
@@ -5120,7 +5020,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="132" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A132" s="2">
         <v>131</v>
       </c>
@@ -5149,7 +5049,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="133" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A133" s="2">
         <v>132</v>
       </c>
@@ -5178,7 +5078,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="134" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A134" s="2">
         <v>133</v>
       </c>
@@ -5207,7 +5107,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="135" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A135" s="2">
         <v>134</v>
       </c>
@@ -5236,7 +5136,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="136" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A136" s="2">
         <v>135</v>
       </c>
@@ -5265,7 +5165,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="137" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A137" s="2">
         <v>136</v>
       </c>
@@ -5294,7 +5194,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="138" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A138" s="2">
         <v>137</v>
       </c>
@@ -5323,7 +5223,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="139" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A139" s="2">
         <v>138</v>
       </c>
@@ -5352,7 +5252,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="140" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A140" s="2">
         <v>139</v>
       </c>
@@ -5381,7 +5281,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="141" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A141" s="2">
         <v>140</v>
       </c>
@@ -5410,7 +5310,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="142" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A142" s="2">
         <v>141</v>
       </c>
@@ -5439,7 +5339,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="143" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A143" s="2">
         <v>142</v>
       </c>
@@ -5468,7 +5368,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="144" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A144" s="2">
         <v>143</v>
       </c>
@@ -5497,7 +5397,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="145" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A145" s="2">
         <v>144</v>
       </c>
@@ -5526,7 +5426,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="146" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A146" s="2">
         <v>145</v>
       </c>
@@ -5555,7 +5455,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="147" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A147" s="2">
         <v>146</v>
       </c>
@@ -5584,7 +5484,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="148" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A148" s="2">
         <v>147</v>
       </c>
@@ -5613,7 +5513,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="149" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A149" s="2">
         <v>148</v>
       </c>
@@ -5642,7 +5542,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="150" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A150" s="2">
         <v>149</v>
       </c>
@@ -5671,7 +5571,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="151" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A151" s="2">
         <v>150</v>
       </c>
@@ -5700,7 +5600,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="152" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A152" s="2">
         <v>151</v>
       </c>
@@ -5729,7 +5629,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="153" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A153" s="2">
         <v>152</v>
       </c>
@@ -5758,7 +5658,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="154" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A154" s="2">
         <v>153</v>
       </c>
@@ -5787,7 +5687,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="155" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A155" s="2">
         <v>154</v>
       </c>
@@ -5816,7 +5716,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="156" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A156" s="2">
         <v>155</v>
       </c>
@@ -5845,7 +5745,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="157" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A157" s="2">
         <v>156</v>
       </c>
@@ -5874,7 +5774,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="158" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A158" s="2">
         <v>157</v>
       </c>
@@ -5903,7 +5803,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="159" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A159" s="2">
         <v>158</v>
       </c>
@@ -5932,7 +5832,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="160" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A160" s="2">
         <v>159</v>
       </c>
@@ -5961,7 +5861,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="161" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A161" s="2">
         <v>160</v>
       </c>
@@ -5990,7 +5890,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="162" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A162" s="2">
         <v>161</v>
       </c>
@@ -6019,7 +5919,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="163" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A163" s="2">
         <v>162</v>
       </c>
@@ -6048,7 +5948,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="164" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A164" s="2">
         <v>163</v>
       </c>
@@ -6077,7 +5977,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="165" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A165" s="2">
         <v>164</v>
       </c>
@@ -6106,7 +6006,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="166" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A166" s="2">
         <v>165</v>
       </c>
@@ -6135,7 +6035,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="167" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A167" s="2">
         <v>166</v>
       </c>
@@ -6164,7 +6064,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="168" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A168" s="2">
         <v>167</v>
       </c>
@@ -6193,7 +6093,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="169" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A169" s="2">
         <v>168</v>
       </c>
@@ -6222,7 +6122,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="170" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A170" s="2">
         <v>169</v>
       </c>
@@ -6251,7 +6151,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="171" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A171" s="2">
         <v>170</v>
       </c>
@@ -6280,7 +6180,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="172" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A172" s="2">
         <v>171</v>
       </c>
@@ -6309,7 +6209,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="173" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A173" s="2">
         <v>172</v>
       </c>
@@ -6338,7 +6238,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="174" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A174" s="2">
         <v>173</v>
       </c>
@@ -6367,7 +6267,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="175" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A175" s="2">
         <v>174</v>
       </c>
@@ -6396,7 +6296,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="176" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A176" s="2">
         <v>175</v>
       </c>
@@ -6425,7 +6325,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="177" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="177" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A177" s="2">
         <v>176</v>
       </c>
@@ -6454,7 +6354,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="178" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="178" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A178" s="2">
         <v>177</v>
       </c>
@@ -6483,7 +6383,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="179" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A179" s="2">
         <v>178</v>
       </c>
@@ -6512,7 +6412,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="180" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="180" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A180" s="2">
         <v>179</v>
       </c>
@@ -6541,7 +6441,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="181" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="181" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A181" s="2">
         <v>180</v>
       </c>
@@ -6570,7 +6470,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="182" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="182" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A182" s="2">
         <v>181</v>
       </c>
@@ -6599,7 +6499,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="183" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="183" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A183" s="2">
         <v>182</v>
       </c>
@@ -6628,7 +6528,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="184" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A184" s="2">
         <v>183</v>
       </c>
@@ -6657,7 +6557,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="185" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="185" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A185" s="2">
         <v>184</v>
       </c>
@@ -6686,7 +6586,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="186" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="186" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A186" s="2">
         <v>185</v>
       </c>
@@ -6715,7 +6615,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="187" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="187" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A187" s="2">
         <v>186</v>
       </c>
@@ -6744,7 +6644,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="188" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="188" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A188" s="2">
         <v>187</v>
       </c>
@@ -6773,7 +6673,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="189" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="189" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A189" s="2">
         <v>188</v>
       </c>
@@ -6802,7 +6702,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="190" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="190" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A190" s="2">
         <v>189</v>
       </c>
@@ -6831,7 +6731,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="191" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="191" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A191" s="2">
         <v>190</v>
       </c>
@@ -6860,7 +6760,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="192" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="192" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A192" s="2">
         <v>191</v>
       </c>
@@ -6889,7 +6789,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="193" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="193" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A193" s="2">
         <v>192</v>
       </c>
@@ -6918,7 +6818,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="194" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="194" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A194" s="2">
         <v>193</v>
       </c>
@@ -6947,7 +6847,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="195" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="195" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A195" s="2">
         <v>194</v>
       </c>
@@ -6976,7 +6876,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="196" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="196" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A196" s="2">
         <v>195</v>
       </c>
@@ -7005,7 +6905,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="197" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="197" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A197" s="2">
         <v>196</v>
       </c>
@@ -7034,7 +6934,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="198" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="198" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A198" s="2">
         <v>197</v>
       </c>
@@ -7063,7 +6963,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="199" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="199" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A199" s="2">
         <v>198</v>
       </c>
@@ -7092,7 +6992,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="200" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="200" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A200" s="2">
         <v>199</v>
       </c>
@@ -7121,7 +7021,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="201" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="201" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A201" s="2">
         <v>200</v>
       </c>
@@ -7150,7 +7050,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="202" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="202" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A202" s="2">
         <v>201</v>
       </c>
@@ -7179,7 +7079,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="203" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="203" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A203" s="2">
         <v>202</v>
       </c>
@@ -7208,7 +7108,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="204" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="204" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A204" s="2">
         <v>203</v>
       </c>
@@ -7237,7 +7137,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="205" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="205" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A205" s="2">
         <v>204</v>
       </c>
@@ -7266,7 +7166,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="206" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="206" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A206" s="2">
         <v>205</v>
       </c>
@@ -7295,7 +7195,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="207" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="207" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A207" s="2">
         <v>206</v>
       </c>
@@ -7324,7 +7224,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="208" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="208" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A208" s="2">
         <v>207</v>
       </c>
@@ -7353,7 +7253,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="209" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="209" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A209" s="2">
         <v>208</v>
       </c>
@@ -7382,7 +7282,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="210" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="210" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A210" s="2">
         <v>209</v>
       </c>
@@ -7411,7 +7311,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="211" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="211" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A211" s="2">
         <v>210</v>
       </c>
@@ -7440,7 +7340,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="212" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="212" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A212" s="2">
         <v>211</v>
       </c>
@@ -7469,7 +7369,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="213" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="213" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A213" s="2">
         <v>212</v>
       </c>
@@ -7498,7 +7398,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="214" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="214" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A214" s="2">
         <v>213</v>
       </c>
@@ -7527,7 +7427,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="215" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="215" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A215" s="2">
         <v>214</v>
       </c>
@@ -7556,7 +7456,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="216" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="216" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A216" s="2">
         <v>215</v>
       </c>
@@ -7585,7 +7485,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="217" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="217" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A217" s="2">
         <v>216</v>
       </c>
@@ -7614,7 +7514,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="218" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="218" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A218" s="2">
         <v>217</v>
       </c>
@@ -7643,7 +7543,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="219" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="219" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A219" s="2">
         <v>218</v>
       </c>
@@ -7672,7 +7572,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="220" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="220" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A220" s="2">
         <v>219</v>
       </c>
@@ -7701,7 +7601,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="221" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="221" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A221" s="2">
         <v>220</v>
       </c>
@@ -7730,7 +7630,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="222" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="222" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A222" s="2">
         <v>221</v>
       </c>
@@ -7759,7 +7659,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="223" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="223" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A223" s="2">
         <v>222</v>
       </c>
@@ -7788,7 +7688,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="224" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="224" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A224" s="2">
         <v>223</v>
       </c>
@@ -7817,7 +7717,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="225" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="225" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A225" s="2">
         <v>224</v>
       </c>
@@ -7846,7 +7746,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="226" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="226" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A226" s="2">
         <v>225</v>
       </c>
@@ -7875,7 +7775,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="227" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="227" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A227" s="2">
         <v>226</v>
       </c>
@@ -7904,7 +7804,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="228" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="228" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A228" s="2">
         <v>227</v>
       </c>
@@ -7933,7 +7833,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="229" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="229" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A229" s="2">
         <v>228</v>
       </c>
@@ -7962,7 +7862,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="230" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="230" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A230" s="2">
         <v>229</v>
       </c>
@@ -7991,7 +7891,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="231" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="231" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A231" s="2">
         <v>230</v>
       </c>
@@ -8020,7 +7920,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="232" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="232" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A232" s="2">
         <v>231</v>
       </c>
@@ -8049,7 +7949,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="233" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="233" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A233" s="2">
         <v>232</v>
       </c>
@@ -8078,7 +7978,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="234" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="234" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A234" s="2">
         <v>233</v>
       </c>
@@ -8107,7 +8007,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="235" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="235" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A235" s="2">
         <v>234</v>
       </c>
@@ -8136,7 +8036,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="236" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="236" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A236" s="2">
         <v>235</v>
       </c>
@@ -8165,7 +8065,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="237" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="237" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A237" s="2">
         <v>236</v>
       </c>
@@ -8194,7 +8094,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="238" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="238" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A238" s="2">
         <v>237</v>
       </c>
@@ -8223,7 +8123,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="239" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="239" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A239" s="2">
         <v>238</v>
       </c>
@@ -8252,7 +8152,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="240" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="240" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A240" s="2">
         <v>239</v>
       </c>
@@ -8281,7 +8181,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="241" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="241" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A241" s="2">
         <v>240</v>
       </c>
@@ -8310,7 +8210,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="242" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="242" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A242" s="2">
         <v>241</v>
       </c>
@@ -8339,7 +8239,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="243" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="243" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A243" s="2">
         <v>242</v>
       </c>
@@ -8368,7 +8268,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="244" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="244" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A244" s="2">
         <v>243</v>
       </c>
@@ -8397,7 +8297,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="245" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="245" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A245" s="2">
         <v>244</v>
       </c>
@@ -8426,7 +8326,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="246" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="246" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A246" s="2">
         <v>245</v>
       </c>
@@ -8455,7 +8355,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="247" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="247" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A247" s="2">
         <v>246</v>
       </c>
@@ -8484,7 +8384,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="248" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="248" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A248" s="2">
         <v>247</v>
       </c>
@@ -8513,7 +8413,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="249" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="249" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A249" s="2">
         <v>248</v>
       </c>
@@ -8542,7 +8442,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="250" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="250" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A250" s="2">
         <v>249</v>
       </c>
@@ -8571,7 +8471,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="251" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="251" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A251" s="2">
         <v>250</v>
       </c>
@@ -8600,7 +8500,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="252" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="252" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A252" s="2">
         <v>251</v>
       </c>
@@ -8629,7 +8529,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="253" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="253" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A253" s="2">
         <v>252</v>
       </c>
@@ -8658,7 +8558,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="254" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="254" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A254" s="2">
         <v>253</v>
       </c>
@@ -8687,7 +8587,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="255" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="255" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A255" s="2">
         <v>254</v>
       </c>
@@ -8716,7 +8616,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="256" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="256" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A256" s="2">
         <v>255</v>
       </c>
@@ -8745,7 +8645,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="257" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="257" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A257" s="2">
         <v>256</v>
       </c>
@@ -8774,7 +8674,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="258" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="258" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A258" s="2">
         <v>257</v>
       </c>
@@ -8803,7 +8703,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="259" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="259" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A259" s="2">
         <v>258</v>
       </c>
@@ -8832,7 +8732,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="260" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="260" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A260" s="2">
         <v>259</v>
       </c>
@@ -8861,7 +8761,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="261" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="261" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A261" s="2">
         <v>260</v>
       </c>
@@ -8890,7 +8790,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="262" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="262" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A262" s="2">
         <v>261</v>
       </c>
@@ -8919,7 +8819,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="263" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="263" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A263" s="2">
         <v>262</v>
       </c>
@@ -8948,7 +8848,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="264" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="264" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A264" s="2">
         <v>263</v>
       </c>
@@ -8977,7 +8877,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="265" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="265" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A265" s="2">
         <v>264</v>
       </c>
@@ -9006,7 +8906,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="266" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="266" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A266" s="2">
         <v>265</v>
       </c>
@@ -9035,7 +8935,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="267" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="267" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A267" s="2">
         <v>266</v>
       </c>
@@ -9064,7 +8964,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="268" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="268" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A268" s="2">
         <v>267</v>
       </c>
@@ -9093,7 +8993,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="269" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="269" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A269" s="2">
         <v>268</v>
       </c>
@@ -9122,7 +9022,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="270" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="270" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A270" s="2">
         <v>269</v>
       </c>
@@ -9151,7 +9051,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="271" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="271" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A271" s="2">
         <v>270</v>
       </c>
@@ -9180,7 +9080,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="272" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="272" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A272" s="2">
         <v>271</v>
       </c>
@@ -9209,7 +9109,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="273" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="273" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A273" s="2">
         <v>272</v>
       </c>
@@ -9238,7 +9138,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="274" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="274" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A274" s="2">
         <v>273</v>
       </c>
@@ -9267,7 +9167,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="275" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="275" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A275" s="2">
         <v>274</v>
       </c>
@@ -9296,7 +9196,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="276" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="276" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A276" s="2">
         <v>275</v>
       </c>
@@ -9325,7 +9225,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="277" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="277" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A277" s="2">
         <v>276</v>
       </c>
@@ -9354,7 +9254,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="278" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="278" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A278" s="2">
         <v>277</v>
       </c>
@@ -9383,7 +9283,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="279" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="279" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A279" s="2">
         <v>278</v>
       </c>
@@ -9412,7 +9312,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="280" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="280" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A280" s="2">
         <v>279</v>
       </c>
@@ -9441,7 +9341,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="281" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="281" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A281" s="2">
         <v>280</v>
       </c>
@@ -9470,7 +9370,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="282" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="282" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A282" s="2">
         <v>281</v>
       </c>
@@ -9499,7 +9399,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="283" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="283" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A283" s="2">
         <v>282</v>
       </c>
@@ -9528,7 +9428,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="284" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="284" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A284" s="2">
         <v>283</v>
       </c>
@@ -9557,7 +9457,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="285" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="285" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A285" s="2">
         <v>284</v>
       </c>
@@ -9586,7 +9486,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="286" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="286" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A286" s="2">
         <v>285</v>
       </c>
@@ -9615,7 +9515,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="287" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="287" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A287" s="2">
         <v>286</v>
       </c>
@@ -9644,7 +9544,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="288" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="288" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A288" s="2">
         <v>287</v>
       </c>
@@ -9673,7 +9573,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="289" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="289" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A289" s="2">
         <v>288</v>
       </c>
@@ -9702,7 +9602,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="290" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="290" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A290" s="2">
         <v>289</v>
       </c>
@@ -9731,7 +9631,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="291" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="291" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A291" s="2">
         <v>290</v>
       </c>
@@ -9760,7 +9660,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="292" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="292" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A292" s="2">
         <v>291</v>
       </c>
@@ -9789,7 +9689,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="293" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="293" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A293" s="2">
         <v>292</v>
       </c>
@@ -9818,7 +9718,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="294" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="294" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A294" s="2">
         <v>293</v>
       </c>
@@ -9847,7 +9747,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="295" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="295" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A295" s="2">
         <v>294</v>
       </c>
@@ -9876,7 +9776,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="296" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="296" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A296" s="2">
         <v>295</v>
       </c>
@@ -9905,7 +9805,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="297" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="297" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A297" s="2">
         <v>296</v>
       </c>
@@ -9934,7 +9834,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="298" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="298" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A298" s="2">
         <v>297</v>
       </c>
@@ -9963,7 +9863,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="299" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="299" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A299" s="2">
         <v>298</v>
       </c>
@@ -9992,7 +9892,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="300" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="300" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A300" s="2">
         <v>299</v>
       </c>
@@ -10021,7 +9921,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="301" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="301" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A301" s="2">
         <v>300</v>
       </c>
@@ -10050,7 +9950,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="302" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="302" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A302" s="2">
         <v>301</v>
       </c>
@@ -10079,7 +9979,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="303" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="303" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A303" s="2">
         <v>302</v>
       </c>
@@ -10108,7 +10008,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="304" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="304" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A304" s="2">
         <v>303</v>
       </c>
@@ -10137,7 +10037,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="305" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="305" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A305" s="2">
         <v>304</v>
       </c>
@@ -10166,7 +10066,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="306" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="306" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A306" s="2">
         <v>305</v>
       </c>
@@ -10195,7 +10095,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="307" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="307" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A307" s="2">
         <v>306</v>
       </c>
@@ -10224,7 +10124,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="308" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="308" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A308" s="2">
         <v>307</v>
       </c>
@@ -10253,7 +10153,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="309" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="309" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A309" s="2">
         <v>308</v>
       </c>
@@ -10282,7 +10182,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="310" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="310" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A310" s="2">
         <v>309</v>
       </c>
@@ -10311,7 +10211,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="311" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="311" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A311" s="2">
         <v>310</v>
       </c>
@@ -10340,7 +10240,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="312" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="312" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A312" s="2">
         <v>311</v>
       </c>
@@ -10369,7 +10269,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="313" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="313" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A313" s="2">
         <v>312</v>
       </c>
@@ -10398,7 +10298,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="314" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="314" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A314" s="2">
         <v>313</v>
       </c>
@@ -10427,7 +10327,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="315" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="315" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A315" s="2">
         <v>314</v>
       </c>
@@ -10456,7 +10356,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="316" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="316" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A316" s="2">
         <v>315</v>
       </c>
@@ -10485,7 +10385,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="317" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="317" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A317" s="2">
         <v>316</v>
       </c>
@@ -10514,7 +10414,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="318" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="318" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A318" s="2">
         <v>317</v>
       </c>
@@ -10543,7 +10443,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="319" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="319" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A319" s="2">
         <v>318</v>
       </c>
@@ -10572,7 +10472,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="320" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="320" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A320" s="2">
         <v>319</v>
       </c>
@@ -10601,7 +10501,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="321" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="321" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A321" s="2">
         <v>320</v>
       </c>
@@ -10630,7 +10530,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="322" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="322" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A322" s="2">
         <v>321</v>
       </c>
@@ -10659,7 +10559,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="323" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="323" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A323" s="2">
         <v>322</v>
       </c>
@@ -10688,7 +10588,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="324" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="324" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A324" s="2">
         <v>323</v>
       </c>
@@ -10717,7 +10617,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="325" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="325" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A325" s="2">
         <v>324</v>
       </c>
@@ -10746,7 +10646,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="326" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="326" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A326" s="2">
         <v>325</v>
       </c>
@@ -10775,7 +10675,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="327" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="327" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A327" s="2">
         <v>326</v>
       </c>
@@ -10804,7 +10704,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="328" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="328" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A328" s="2">
         <v>327</v>
       </c>
@@ -10833,7 +10733,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="329" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="329" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A329" s="2">
         <v>328</v>
       </c>
@@ -10862,7 +10762,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="330" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="330" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A330" s="2">
         <v>329</v>
       </c>
@@ -10891,7 +10791,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="331" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="331" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A331" s="2">
         <v>330</v>
       </c>
@@ -10920,7 +10820,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="332" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="332" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A332" s="2">
         <v>331</v>
       </c>
@@ -10949,7 +10849,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="333" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="333" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A333" s="2">
         <v>332</v>
       </c>
@@ -10978,7 +10878,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="334" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="334" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A334" s="2">
         <v>333</v>
       </c>
@@ -11007,7 +10907,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="335" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="335" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A335" s="2">
         <v>334</v>
       </c>
@@ -11036,7 +10936,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="336" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="336" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A336" s="2">
         <v>335</v>
       </c>
@@ -11065,7 +10965,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="337" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="337" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A337" s="2">
         <v>336</v>
       </c>
@@ -11094,7 +10994,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="338" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="338" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A338" s="2">
         <v>337</v>
       </c>
@@ -11123,7 +11023,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="339" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="339" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A339" s="2">
         <v>338</v>
       </c>
@@ -11152,7 +11052,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="340" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="340" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A340" s="2">
         <v>339</v>
       </c>
@@ -11181,7 +11081,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="341" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="341" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A341" s="2">
         <v>340</v>
       </c>
@@ -11210,7 +11110,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="342" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="342" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A342" s="2">
         <v>341</v>
       </c>
@@ -11239,7 +11139,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="343" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="343" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A343" s="2">
         <v>342</v>
       </c>
@@ -11268,7 +11168,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="344" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="344" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A344" s="2">
         <v>343</v>
       </c>
@@ -11297,7 +11197,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="345" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="345" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A345" s="2">
         <v>344</v>
       </c>
@@ -11326,7 +11226,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="346" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="346" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A346" s="2">
         <v>345</v>
       </c>
@@ -11355,7 +11255,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="347" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="347" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A347" s="2">
         <v>346</v>
       </c>
@@ -11384,7 +11284,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="348" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="348" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A348" s="2">
         <v>347</v>
       </c>
@@ -11413,7 +11313,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="349" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="349" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A349" s="2">
         <v>348</v>
       </c>
@@ -11442,7 +11342,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="350" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="350" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A350" s="2">
         <v>349</v>
       </c>
@@ -11471,7 +11371,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="351" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="351" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A351" s="2">
         <v>350</v>
       </c>
@@ -11500,7 +11400,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="352" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="352" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A352" s="2">
         <v>351</v>
       </c>
@@ -11529,7 +11429,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="353" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="353" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A353" s="2">
         <v>352</v>
       </c>
@@ -11558,7 +11458,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="354" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="354" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A354" s="2">
         <v>353</v>
       </c>
@@ -11587,7 +11487,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="355" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="355" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A355" s="2">
         <v>354</v>
       </c>
@@ -11616,7 +11516,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="356" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="356" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A356" s="2">
         <v>355</v>
       </c>
@@ -11645,7 +11545,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="357" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="357" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A357" s="2">
         <v>356</v>
       </c>
@@ -11674,7 +11574,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="358" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="358" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A358" s="2">
         <v>357</v>
       </c>
@@ -11703,7 +11603,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="359" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="359" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A359" s="2">
         <v>358</v>
       </c>
@@ -11732,7 +11632,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="360" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="360" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A360" s="2">
         <v>359</v>
       </c>
@@ -11761,7 +11661,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="361" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="361" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A361" s="2">
         <v>360</v>
       </c>
@@ -11790,7 +11690,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="362" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="362" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A362" s="2">
         <v>361</v>
       </c>
@@ -11819,7 +11719,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="363" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="363" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A363" s="2">
         <v>362</v>
       </c>
@@ -11848,7 +11748,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="364" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="364" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A364" s="2">
         <v>363</v>
       </c>
@@ -11877,7 +11777,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="365" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="365" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A365" s="2">
         <v>364</v>
       </c>
@@ -11906,7 +11806,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="366" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="366" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A366" s="2">
         <v>365</v>
       </c>
@@ -11935,7 +11835,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="367" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="367" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A367" s="2">
         <v>366</v>
       </c>
@@ -11964,7 +11864,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="368" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="368" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A368" s="2">
         <v>367</v>
       </c>
@@ -11993,7 +11893,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="369" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="369" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A369" s="2">
         <v>368</v>
       </c>
@@ -12022,7 +11922,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="370" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="370" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A370" s="2">
         <v>369</v>
       </c>
@@ -12051,7 +11951,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="371" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="371" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A371" s="2">
         <v>370</v>
       </c>
@@ -12080,7 +11980,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="372" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="372" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A372" s="2">
         <v>371</v>
       </c>
@@ -12109,7 +12009,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="373" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="373" spans="1:9" ht="16" x14ac:dyDescent="0.35">
       <c r="A373" s="2">
         <v>372</v>
       </c>
@@ -12140,6 +12040,5 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>